<commit_message>
Add Digital продюсер Иманбаева to Marcom across all outputs
Add the missing position (Иманбаева Аяулым Маратовна, Digital продюсер,
1 000 162 ₸) to Marcom's «Промо / Контент» block in the Excel source, the
PowerPoint deck, and the self-updating HTML. Marcom is now 14 people;
department ФОТ and the grand total (44 050 321 ₸) recompute accordingly.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015FvdqNtbbJPjugTChUgZkw
</commit_message>
<xml_diff>
--- a/Данные — структура и ФОТ.xlsx
+++ b/Данные — структура и ФОТ.xlsx
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -918,7 +918,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>SMM</t>
+          <t>Промо / Контент</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -928,22 +928,22 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Head of SMM · Мария</t>
+          <t>Promo · Аяулым</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Коренькова Мария Николаевна</t>
+          <t>Иманбаева Аяулым Маратовна</t>
         </is>
       </c>
       <c r="G9" s="8" t="n">
-        <v>1625032</v>
+        <v>1000162</v>
       </c>
       <c r="H9" s="9" t="inlineStr"/>
       <c r="I9" s="9" t="inlineStr"/>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>M_SMM_1</t>
+          <t>M_PROMO_6</t>
         </is>
       </c>
     </row>
@@ -968,26 +968,22 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>SMM Original</t>
+          <t>Head of SMM · Мария</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>SMM менеджер · имя н/д</t>
-        </is>
-      </c>
-      <c r="G10" s="10" t="n">
-        <v>867456</v>
-      </c>
-      <c r="H10" s="9" t="inlineStr">
-        <is>
-          <t>макс.</t>
-        </is>
-      </c>
+          <t>Коренькова Мария Николаевна</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>1625032</v>
+      </c>
+      <c r="H10" s="9" t="inlineStr"/>
       <c r="I10" s="9" t="inlineStr"/>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>M_SMM_2</t>
+          <t>M_SMM_1</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1008,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>SMM Gen</t>
+          <t>SMM Original</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -1031,7 +1027,7 @@
       <c r="I11" s="9" t="inlineStr"/>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>M_SMM_3</t>
+          <t>M_SMM_2</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1052,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>SMM Sport</t>
+          <t>SMM Gen</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -1075,7 +1071,7 @@
       <c r="I12" s="9" t="inlineStr"/>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>M_SMM_4</t>
+          <t>M_SMM_3</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1096,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>SMM Original</t>
+          <t>SMM Sport</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -1119,7 +1115,7 @@
       <c r="I13" s="9" t="inlineStr"/>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>M_SMM_5</t>
+          <t>M_SMM_4</t>
         </is>
       </c>
     </row>
@@ -1144,22 +1140,26 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Telegram редактор Sport</t>
+          <t>SMM Original</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Куричев Иван Николаевич</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="n">
-        <v>513920</v>
-      </c>
-      <c r="H14" s="9" t="inlineStr"/>
+          <t>SMM менеджер · имя н/д</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>867456</v>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>макс.</t>
+        </is>
+      </c>
       <c r="I14" s="9" t="inlineStr"/>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>M_SMM_6</t>
+          <t>M_SMM_5</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1174,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>SMM</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1184,22 +1184,22 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Pr manager · Аружан</t>
+          <t>Telegram редактор Sport</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>PR менеджер</t>
+          <t>Куричев Иван Николаевич</t>
         </is>
       </c>
       <c r="G15" s="8" t="n">
-        <v>1212314</v>
+        <v>513920</v>
       </c>
       <c r="H15" s="9" t="inlineStr"/>
       <c r="I15" s="9" t="inlineStr"/>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>M_PR_1</t>
+          <t>M_SMM_6</t>
         </is>
       </c>
     </row>
@@ -1209,37 +1209,37 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Каналы коммуникации</t>
+          <t>Marcom</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Руководитель</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Руководитель</t>
+          <t>Сотрудник</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Head · Эдуард Д</t>
+          <t>Pr manager · Аружан</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Head каналы коммуникации</t>
+          <t>PR менеджер</t>
         </is>
       </c>
       <c r="G16" s="8" t="n">
-        <v>2260000</v>
+        <v>1212314</v>
       </c>
       <c r="H16" s="9" t="inlineStr"/>
       <c r="I16" s="9" t="inlineStr"/>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>K_HEAD</t>
+          <t>M_PR_1</t>
         </is>
       </c>
     </row>
@@ -1254,32 +1254,32 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Руководитель</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Сотрудник</t>
+          <t>Руководитель</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Senior PPC · Антон Б</t>
+          <t>Head · Эдуард Д</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Senior PPC</t>
+          <t>Head каналы коммуникации</t>
         </is>
       </c>
       <c r="G17" s="8" t="n">
-        <v>1346342</v>
+        <v>2260000</v>
       </c>
       <c r="H17" s="9" t="inlineStr"/>
       <c r="I17" s="9" t="inlineStr"/>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>K_1</t>
+          <t>K_HEAD</t>
         </is>
       </c>
     </row>
@@ -1304,22 +1304,22 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Media manager · Халмурад</t>
+          <t>Senior PPC · Антон Б</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Медиа менеджер</t>
+          <t>Senior PPC</t>
         </is>
       </c>
       <c r="G18" s="8" t="n">
-        <v>1056850</v>
+        <v>1346342</v>
       </c>
       <c r="H18" s="9" t="inlineStr"/>
       <c r="I18" s="9" t="inlineStr"/>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>K_2</t>
+          <t>K_1</t>
         </is>
       </c>
     </row>
@@ -1344,22 +1344,22 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Внут. маркетинг · Аида Е</t>
+          <t>Media manager · Халмурад</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Внутренний маркетинг</t>
+          <t>Медиа менеджер</t>
         </is>
       </c>
       <c r="G19" s="8" t="n">
-        <v>1058434</v>
+        <v>1056850</v>
       </c>
       <c r="H19" s="9" t="inlineStr"/>
       <c r="I19" s="9" t="inlineStr"/>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>K_3</t>
+          <t>K_2</t>
         </is>
       </c>
     </row>
@@ -1384,114 +1384,114 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>PPC (1)</t>
+          <t>Внут. маркетинг · Аида Е</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Трафик менеджер · имя н/д</t>
-        </is>
-      </c>
-      <c r="G20" s="10" t="n">
-        <v>1124000</v>
-      </c>
-      <c r="H20" s="9" t="inlineStr">
-        <is>
-          <t>макс.</t>
-        </is>
-      </c>
+          <t>Внутренний маркетинг</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>1058434</v>
+      </c>
+      <c r="H20" s="9" t="inlineStr"/>
       <c r="I20" s="9" t="inlineStr"/>
       <c r="J20" s="5" t="inlineStr">
         <is>
+          <t>K_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Каналы коммуникации</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Сотрудник</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>PPC (1)</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Трафик менеджер · имя н/д</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="n">
+        <v>1124000</v>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>макс.</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr"/>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
           <t>K_4</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="11" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>Каналы коммуникации</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
+      <c r="C22" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>Сотрудник</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>Сотрудник</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
         <is>
           <t>CVM (?)</t>
         </is>
       </c>
-      <c r="F21" s="15" t="inlineStr">
+      <c r="F22" s="15" t="inlineStr">
         <is>
           <t>CRM менеджер · планируется</t>
         </is>
       </c>
-      <c r="G21" s="16" t="n">
+      <c r="G22" s="16" t="n">
         <v>867456</v>
       </c>
-      <c r="H21" s="17" t="inlineStr">
+      <c r="H22" s="17" t="inlineStr">
         <is>
           <t>макс.</t>
         </is>
       </c>
-      <c r="I21" s="17" t="inlineStr">
+      <c r="I22" s="17" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="J21" s="13" t="inlineStr">
+      <c r="J22" s="13" t="inlineStr">
         <is>
           <t>K_5</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Продакшн</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Руководитель</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Руководитель</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>Head of creative · Катерина Р</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>Креативный директор</t>
-        </is>
-      </c>
-      <c r="G22" s="8" t="n">
-        <v>2490895</v>
-      </c>
-      <c r="H22" s="9" t="inlineStr"/>
-      <c r="I22" s="9" t="inlineStr"/>
-      <c r="J22" s="5" t="inlineStr">
-        <is>
-          <t>P_HEAD</t>
         </is>
       </c>
     </row>
@@ -1506,32 +1506,32 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Арт</t>
+          <t>Руководитель</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Суб-лид</t>
+          <t>Руководитель</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Senior art · Олег Н</t>
+          <t>Head of creative · Катерина Р</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Назаренко Олег Станиславович</t>
+          <t>Креативный директор</t>
         </is>
       </c>
       <c r="G23" s="8" t="n">
-        <v>1494981</v>
+        <v>2490895</v>
       </c>
       <c r="H23" s="9" t="inlineStr"/>
       <c r="I23" s="9" t="inlineStr"/>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>P_ART</t>
+          <t>P_HEAD</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Продакшн</t>
+          <t>Арт</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -1556,22 +1556,22 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Senior production · Александр Е</t>
+          <t>Senior art · Олег Н</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>Senior production</t>
+          <t>Назаренко Олег Станиславович</t>
         </is>
       </c>
       <c r="G24" s="8" t="n">
-        <v>1291685</v>
+        <v>1494981</v>
       </c>
       <c r="H24" s="9" t="inlineStr"/>
       <c r="I24" s="9" t="inlineStr"/>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>P_PROD</t>
+          <t>P_ART</t>
         </is>
       </c>
     </row>
@@ -1586,36 +1586,32 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Арт</t>
+          <t>Продакшн</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Сотрудник</t>
+          <t>Суб-лид</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Graph</t>
+          <t>Senior production · Александр Е</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Дизайнер · имя н/д</t>
-        </is>
-      </c>
-      <c r="G25" s="10" t="n">
-        <v>940000</v>
-      </c>
-      <c r="H25" s="9" t="inlineStr">
-        <is>
-          <t>макс.</t>
-        </is>
-      </c>
+          <t>Senior production</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="n">
+        <v>1291685</v>
+      </c>
+      <c r="H25" s="9" t="inlineStr"/>
       <c r="I25" s="9" t="inlineStr"/>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>P_ART_1</t>
+          <t>P_PROD</t>
         </is>
       </c>
     </row>
@@ -1659,7 +1655,7 @@
       <c r="I26" s="9" t="inlineStr"/>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>P_ART_2</t>
+          <t>P_ART_1</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1680,7 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Graph Спорт</t>
+          <t>Graph</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
@@ -1703,7 +1699,7 @@
       <c r="I27" s="9" t="inlineStr"/>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>P_ART_3</t>
+          <t>P_ART_2</t>
         </is>
       </c>
     </row>
@@ -1728,16 +1724,16 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Graph Спорт</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>Motion-дизайнер · имя н/д</t>
+          <t>Дизайнер · имя н/д</t>
         </is>
       </c>
       <c r="G28" s="10" t="n">
-        <v>877000</v>
+        <v>940000</v>
       </c>
       <c r="H28" s="9" t="inlineStr">
         <is>
@@ -1747,7 +1743,7 @@
       <c r="I28" s="9" t="inlineStr"/>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>P_ART_4</t>
+          <t>P_ART_3</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1787,7 @@
       <c r="I29" s="9" t="inlineStr"/>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>P_ART_5</t>
+          <t>P_ART_4</t>
         </is>
       </c>
     </row>
@@ -1806,7 +1802,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Продакшн</t>
+          <t>Арт</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -1816,16 +1812,16 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Мобилограф / монтажёр</t>
+          <t>Motion</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>Видеограф · имя н/д</t>
+          <t>Motion-дизайнер · имя н/д</t>
         </is>
       </c>
       <c r="G30" s="10" t="n">
-        <v>1498769</v>
+        <v>877000</v>
       </c>
       <c r="H30" s="9" t="inlineStr">
         <is>
@@ -1835,7 +1831,7 @@
       <c r="I30" s="9" t="inlineStr"/>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>P_PROD_1</t>
+          <t>P_ART_5</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1875,7 @@
       <c r="I31" s="9" t="inlineStr"/>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>P_PROD_2</t>
+          <t>P_PROD_1</t>
         </is>
       </c>
     </row>
@@ -1923,7 +1919,7 @@
       <c r="I32" s="9" t="inlineStr"/>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>P_PROD_3</t>
+          <t>P_PROD_2</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1944,7 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Мобилограф / монтажёр Sport</t>
+          <t>Мобилограф / монтажёр</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
@@ -1967,7 +1963,7 @@
       <c r="I33" s="9" t="inlineStr"/>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>P_PROD_4</t>
+          <t>P_PROD_3</t>
         </is>
       </c>
     </row>
@@ -1977,37 +1973,41 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Проджект</t>
+          <t>Продакшн</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Руководитель</t>
+          <t>Продакшн</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Руководитель</t>
+          <t>Сотрудник</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Head · Ольга М</t>
+          <t>Мобилограф / монтажёр Sport</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>Head project</t>
-        </is>
-      </c>
-      <c r="G34" s="8" t="n">
-        <v>1291685</v>
-      </c>
-      <c r="H34" s="9" t="inlineStr"/>
+          <t>Видеограф · имя н/д</t>
+        </is>
+      </c>
+      <c r="G34" s="10" t="n">
+        <v>1498769</v>
+      </c>
+      <c r="H34" s="9" t="inlineStr">
+        <is>
+          <t>макс.</t>
+        </is>
+      </c>
       <c r="I34" s="9" t="inlineStr"/>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>PJ_HEAD</t>
+          <t>P_PROD_4</t>
         </is>
       </c>
     </row>
@@ -2022,32 +2022,32 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Руководитель</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Сотрудник</t>
+          <t>Руководитель</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Project manager · Аружан С</t>
+          <t>Head · Ольга М</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Проджект-менеджер</t>
+          <t>Head project</t>
         </is>
       </c>
       <c r="G35" s="8" t="n">
-        <v>700000</v>
+        <v>1291685</v>
       </c>
       <c r="H35" s="9" t="inlineStr"/>
       <c r="I35" s="9" t="inlineStr"/>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>PJ_1</t>
+          <t>PJ_HEAD</t>
         </is>
       </c>
     </row>
@@ -2072,22 +2072,22 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Project manager · Анель</t>
+          <t>Project manager · Аружан С</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>Муханова Анель Султановна</t>
+          <t>Проджект-менеджер</t>
         </is>
       </c>
       <c r="G36" s="8" t="n">
-        <v>741192</v>
+        <v>700000</v>
       </c>
       <c r="H36" s="9" t="inlineStr"/>
       <c r="I36" s="9" t="inlineStr"/>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>PJ_2</t>
+          <t>PJ_1</t>
         </is>
       </c>
     </row>
@@ -2112,22 +2112,22 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Спецпроекты · Марина</t>
+          <t>Project manager · Анель</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Гяурова Марина Якубовна</t>
+          <t>Муханова Анель Султановна</t>
         </is>
       </c>
       <c r="G37" s="8" t="n">
-        <v>1000162</v>
+        <v>741192</v>
       </c>
       <c r="H37" s="9" t="inlineStr"/>
       <c r="I37" s="9" t="inlineStr"/>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>PJ_3</t>
+          <t>PJ_2</t>
         </is>
       </c>
     </row>
@@ -2152,27 +2152,67 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>B2B и продакшн · Олеся М</t>
+          <t>Спецпроекты · Марина</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>B2B и продакшн</t>
+          <t>Гяурова Марина Якубовна</t>
         </is>
       </c>
       <c r="G38" s="8" t="n">
-        <v>1081000</v>
+        <v>1000162</v>
       </c>
       <c r="H38" s="9" t="inlineStr"/>
       <c r="I38" s="9" t="inlineStr"/>
       <c r="J38" s="5" t="inlineStr">
         <is>
+          <t>PJ_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Проджект</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Сотрудник</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>B2B и продакшн · Олеся М</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>B2B и продакшн</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="n">
+        <v>1081000</v>
+      </c>
+      <c r="H39" s="9" t="inlineStr"/>
+      <c r="I39" s="9" t="inlineStr"/>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
           <t>PJ_4</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="18" t="inlineStr">
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="18" t="inlineStr">
         <is>
           <t>Синие ячейки в «Оклад, ₸» — редактируемые. «Признак: макс.» — имя на позиции не определено, подставлена максимальная стоимость по позиции. «Вакансия: да» — планируемая позиция. Итоги считаются на листе «Свод».</t>
         </is>
@@ -2180,8 +2220,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A40:J40"/>
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A41:J41"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2232,11 +2272,11 @@
         </is>
       </c>
       <c r="B3" s="22">
-        <f>COUNTIF(Данные!$B$3:$B$38,A3)</f>
+        <f>COUNTIF(Данные!$B$3:$B$39,A3)</f>
         <v/>
       </c>
       <c r="C3" s="23">
-        <f>SUMIF(Данные!$B$3:$B$38,A3,Данные!$G$3:$G$38)</f>
+        <f>SUMIF(Данные!$B$3:$B$39,A3,Данные!$G$3:$G$39)</f>
         <v/>
       </c>
     </row>
@@ -2247,11 +2287,11 @@
         </is>
       </c>
       <c r="B4" s="25">
-        <f>COUNTIF(Данные!$B$3:$B$38,A4)</f>
+        <f>COUNTIF(Данные!$B$3:$B$39,A4)</f>
         <v/>
       </c>
       <c r="C4" s="26">
-        <f>SUMIF(Данные!$B$3:$B$38,A4,Данные!$G$3:$G$38)</f>
+        <f>SUMIF(Данные!$B$3:$B$39,A4,Данные!$G$3:$G$39)</f>
         <v/>
       </c>
     </row>
@@ -2262,11 +2302,11 @@
         </is>
       </c>
       <c r="B5" s="22">
-        <f>COUNTIF(Данные!$B$3:$B$38,A5)</f>
+        <f>COUNTIF(Данные!$B$3:$B$39,A5)</f>
         <v/>
       </c>
       <c r="C5" s="23">
-        <f>SUMIF(Данные!$B$3:$B$38,A5,Данные!$G$3:$G$38)</f>
+        <f>SUMIF(Данные!$B$3:$B$39,A5,Данные!$G$3:$G$39)</f>
         <v/>
       </c>
     </row>
@@ -2277,11 +2317,11 @@
         </is>
       </c>
       <c r="B6" s="25">
-        <f>COUNTIF(Данные!$B$3:$B$38,A6)</f>
+        <f>COUNTIF(Данные!$B$3:$B$39,A6)</f>
         <v/>
       </c>
       <c r="C6" s="26">
-        <f>SUMIF(Данные!$B$3:$B$38,A6,Данные!$G$3:$G$38)</f>
+        <f>SUMIF(Данные!$B$3:$B$39,A6,Данные!$G$3:$G$39)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Match original screens: split by direction + real монтажёр names
Rework Marcom and Продакшн layouts to mirror the source screenshots:
- Marcom: Контент in two columns, SMM split into parallel Originals/Gen/
  Sport columns under Head of SMM, PR on the right.
- Продакшн: Design branch (Graph + Motion columns) under Senior art and
  Video production branch under Senior production.
Fill the four Мобилограф/монтажёр boxes with the real production
videographers and their salaries (Асанов 1 000 162, Шаймардан 751 000,
Жұмағали 804 324, Боровков/Sport 523 000), dropping the max-cost
placeholder. Продакшн ФОТ recomputes to 12 930 047 ₸; grand total
41 133 731 ₸. Applied across Excel, PowerPoint and the HTML presentation.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015FvdqNtbbJPjugTChUgZkw
</commit_message>
<xml_diff>
--- a/Данные — структура и ФОТ.xlsx
+++ b/Данные — структура и ФОТ.xlsx
@@ -1861,17 +1861,13 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Видеограф · имя н/д</t>
-        </is>
-      </c>
-      <c r="G31" s="10" t="n">
-        <v>1498769</v>
-      </c>
-      <c r="H31" s="9" t="inlineStr">
-        <is>
-          <t>макс.</t>
-        </is>
-      </c>
+          <t>Асанов Әділ Асанұлы</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="n">
+        <v>1000162</v>
+      </c>
+      <c r="H31" s="9" t="inlineStr"/>
       <c r="I31" s="9" t="inlineStr"/>
       <c r="J31" s="5" t="inlineStr">
         <is>
@@ -1905,17 +1901,13 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>Видеограф · имя н/д</t>
-        </is>
-      </c>
-      <c r="G32" s="10" t="n">
-        <v>1498769</v>
-      </c>
-      <c r="H32" s="9" t="inlineStr">
-        <is>
-          <t>макс.</t>
-        </is>
-      </c>
+          <t>Шаймардан Мағжан Адилұлы</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="n">
+        <v>751000</v>
+      </c>
+      <c r="H32" s="9" t="inlineStr"/>
       <c r="I32" s="9" t="inlineStr"/>
       <c r="J32" s="5" t="inlineStr">
         <is>
@@ -1949,17 +1941,13 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Видеограф · имя н/д</t>
-        </is>
-      </c>
-      <c r="G33" s="10" t="n">
-        <v>1498769</v>
-      </c>
-      <c r="H33" s="9" t="inlineStr">
-        <is>
-          <t>макс.</t>
-        </is>
-      </c>
+          <t>Жұмағали Әділжан Бауыржанұлы</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>804324</v>
+      </c>
+      <c r="H33" s="9" t="inlineStr"/>
       <c r="I33" s="9" t="inlineStr"/>
       <c r="J33" s="5" t="inlineStr">
         <is>
@@ -1993,17 +1981,13 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>Видеограф · имя н/д</t>
-        </is>
-      </c>
-      <c r="G34" s="10" t="n">
-        <v>1498769</v>
-      </c>
-      <c r="H34" s="9" t="inlineStr">
-        <is>
-          <t>макс.</t>
-        </is>
-      </c>
+          <t>Боровков Владимир Владимирович</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="n">
+        <v>523000</v>
+      </c>
+      <c r="H34" s="9" t="inlineStr"/>
       <c r="I34" s="9" t="inlineStr"/>
       <c r="J34" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix Video production: remove Боровков, tag real videographers by direction
Боровков was not part of the team — remove him everywhere. Video
production now lists the three actual videographers with their directions:
Асанов Әділ (Originals, 1 000 162), Шаймардан Мағжан (Originals, 751 000)
and Жұмағали Әділжан (Sport, 804 324). Продакшн is now 11 people, ФОТ
12 407 047 ₸; grand total 40 610 731 ₸. Applied to Excel, PowerPoint, HTML.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015FvdqNtbbJPjugTChUgZkw
</commit_message>
<xml_diff>
--- a/Данные — структура и ФОТ.xlsx
+++ b/Данные — структура и ФОТ.xlsx
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Асанов Әділ Асанұлы</t>
+          <t>Асанов Әділ · Originals</t>
         </is>
       </c>
       <c r="G31" s="8" t="n">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>Шаймардан Мағжан Адилұлы</t>
+          <t>Шаймардан Мағжан · Originals</t>
         </is>
       </c>
       <c r="G32" s="8" t="n">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Жұмағали Әділжан Бауыржанұлы</t>
+          <t>Жұмағали Әділжан · Sport</t>
         </is>
       </c>
       <c r="G33" s="8" t="n">
@@ -1961,37 +1961,37 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Продакшн</t>
+          <t>Проджект</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Продакшн</t>
+          <t>Руководитель</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Сотрудник</t>
+          <t>Руководитель</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Мобилограф / монтажёр Sport</t>
+          <t>Head · Ольга М</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>Боровков Владимир Владимирович</t>
+          <t>Head project</t>
         </is>
       </c>
       <c r="G34" s="8" t="n">
-        <v>523000</v>
+        <v>1291685</v>
       </c>
       <c r="H34" s="9" t="inlineStr"/>
       <c r="I34" s="9" t="inlineStr"/>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>P_PROD_4</t>
+          <t>PJ_HEAD</t>
         </is>
       </c>
     </row>
@@ -2006,32 +2006,32 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Руководитель</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Руководитель</t>
+          <t>Сотрудник</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Head · Ольга М</t>
+          <t>Project manager · Аружан С</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Head project</t>
+          <t>Проджект-менеджер</t>
         </is>
       </c>
       <c r="G35" s="8" t="n">
-        <v>1291685</v>
+        <v>700000</v>
       </c>
       <c r="H35" s="9" t="inlineStr"/>
       <c r="I35" s="9" t="inlineStr"/>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>PJ_HEAD</t>
+          <t>PJ_1</t>
         </is>
       </c>
     </row>
@@ -2056,22 +2056,22 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Project manager · Аружан С</t>
+          <t>Project manager · Анель</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>Проджект-менеджер</t>
+          <t>Муханова Анель Султановна</t>
         </is>
       </c>
       <c r="G36" s="8" t="n">
-        <v>700000</v>
+        <v>741192</v>
       </c>
       <c r="H36" s="9" t="inlineStr"/>
       <c r="I36" s="9" t="inlineStr"/>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>PJ_1</t>
+          <t>PJ_2</t>
         </is>
       </c>
     </row>
@@ -2096,22 +2096,22 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Project manager · Анель</t>
+          <t>Спецпроекты · Марина</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Муханова Анель Султановна</t>
+          <t>Гяурова Марина Якубовна</t>
         </is>
       </c>
       <c r="G37" s="8" t="n">
-        <v>741192</v>
+        <v>1000162</v>
       </c>
       <c r="H37" s="9" t="inlineStr"/>
       <c r="I37" s="9" t="inlineStr"/>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>PJ_2</t>
+          <t>PJ_3</t>
         </is>
       </c>
     </row>
@@ -2136,67 +2136,27 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Спецпроекты · Марина</t>
+          <t>B2B и продакшн · Олеся М</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>Гяурова Марина Якубовна</t>
+          <t>B2B и продакшн</t>
         </is>
       </c>
       <c r="G38" s="8" t="n">
-        <v>1000162</v>
+        <v>1081000</v>
       </c>
       <c r="H38" s="9" t="inlineStr"/>
       <c r="I38" s="9" t="inlineStr"/>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>PJ_3</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="n">
-        <v>37</v>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>Проджект</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Сотрудник</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="inlineStr">
-        <is>
-          <t>B2B и продакшн · Олеся М</t>
-        </is>
-      </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>B2B и продакшн</t>
-        </is>
-      </c>
-      <c r="G39" s="8" t="n">
-        <v>1081000</v>
-      </c>
-      <c r="H39" s="9" t="inlineStr"/>
-      <c r="I39" s="9" t="inlineStr"/>
-      <c r="J39" s="5" t="inlineStr">
-        <is>
           <t>PJ_4</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="18" t="inlineStr">
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="18" t="inlineStr">
         <is>
           <t>Синие ячейки в «Оклад, ₸» — редактируемые. «Признак: макс.» — имя на позиции не определено, подставлена максимальная стоимость по позиции. «Вакансия: да» — планируемая позиция. Итоги считаются на листе «Свод».</t>
         </is>
@@ -2204,8 +2164,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A40:J40"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A41:J41"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2256,11 +2216,11 @@
         </is>
       </c>
       <c r="B3" s="22">
-        <f>COUNTIF(Данные!$B$3:$B$39,A3)</f>
+        <f>COUNTIF(Данные!$B$3:$B$38,A3)</f>
         <v/>
       </c>
       <c r="C3" s="23">
-        <f>SUMIF(Данные!$B$3:$B$39,A3,Данные!$G$3:$G$39)</f>
+        <f>SUMIF(Данные!$B$3:$B$38,A3,Данные!$G$3:$G$38)</f>
         <v/>
       </c>
     </row>
@@ -2271,11 +2231,11 @@
         </is>
       </c>
       <c r="B4" s="25">
-        <f>COUNTIF(Данные!$B$3:$B$39,A4)</f>
+        <f>COUNTIF(Данные!$B$3:$B$38,A4)</f>
         <v/>
       </c>
       <c r="C4" s="26">
-        <f>SUMIF(Данные!$B$3:$B$39,A4,Данные!$G$3:$G$39)</f>
+        <f>SUMIF(Данные!$B$3:$B$38,A4,Данные!$G$3:$G$38)</f>
         <v/>
       </c>
     </row>
@@ -2286,11 +2246,11 @@
         </is>
       </c>
       <c r="B5" s="22">
-        <f>COUNTIF(Данные!$B$3:$B$39,A5)</f>
+        <f>COUNTIF(Данные!$B$3:$B$38,A5)</f>
         <v/>
       </c>
       <c r="C5" s="23">
-        <f>SUMIF(Данные!$B$3:$B$39,A5,Данные!$G$3:$G$39)</f>
+        <f>SUMIF(Данные!$B$3:$B$38,A5,Данные!$G$3:$G$38)</f>
         <v/>
       </c>
     </row>
@@ -2301,11 +2261,11 @@
         </is>
       </c>
       <c r="B6" s="25">
-        <f>COUNTIF(Данные!$B$3:$B$39,A6)</f>
+        <f>COUNTIF(Данные!$B$3:$B$38,A6)</f>
         <v/>
       </c>
       <c r="C6" s="26">
-        <f>SUMIF(Данные!$B$3:$B$39,A6,Данные!$G$3:$G$39)</f>
+        <f>SUMIF(Данные!$B$3:$B$38,A6,Данные!$G$3:$G$38)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync real names from user's edited PDF; swap Боровков for Жанабеков
Bring the source in line with the user's edited export: fill in the real
SMM names (Шафкат Дария, Жандильдина Сабина, Шакрат Темірлан, Кулбаева
Салтанат) and design names (Ахметова, Ли Яна, Аркениязов, Мкпо Майкл, plus
a «Граф дизайнер» placeholder), and set the Senior production subtitle.
Per instruction, replace Боровков with Жанабеков Кудайберген (1 498 769) in
Video production. Marcom 15 496 844 ₸, Продакшн 13 581 877 ₸ (12 people),
grand total 41 605 842 ₸. Applied to Excel, PowerPoint and HTML.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015FvdqNtbbJPjugTChUgZkw
</commit_message>
<xml_diff>
--- a/Данные — структура и ФОТ.xlsx
+++ b/Данные — структура и ФОТ.xlsx
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1013,17 +1013,13 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>SMM менеджер · имя н/д</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="n">
-        <v>867456</v>
-      </c>
-      <c r="H11" s="9" t="inlineStr">
-        <is>
-          <t>макс.</t>
-        </is>
-      </c>
+          <t>Шафкат Дария</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>741193</v>
+      </c>
+      <c r="H11" s="9" t="inlineStr"/>
       <c r="I11" s="9" t="inlineStr"/>
       <c r="J11" s="5" t="inlineStr">
         <is>
@@ -1057,17 +1053,13 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>SMM менеджер · имя н/д</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="n">
-        <v>867456</v>
-      </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>макс.</t>
-        </is>
-      </c>
+          <t>Жандильдина Сабина Канатовна</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>814000</v>
+      </c>
+      <c r="H12" s="9" t="inlineStr"/>
       <c r="I12" s="9" t="inlineStr"/>
       <c r="J12" s="5" t="inlineStr">
         <is>
@@ -1101,7 +1093,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>SMM менеджер · имя н/д</t>
+          <t>Шакрат Темірлан Талғатұлы</t>
         </is>
       </c>
       <c r="G13" s="10" t="n">
@@ -1145,7 +1137,7 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>SMM менеджер · имя н/д</t>
+          <t>Кулбаева Салтанат Фархатқызы</t>
         </is>
       </c>
       <c r="G14" s="10" t="n">
@@ -1601,7 +1593,7 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Senior production</t>
+          <t>Александр Е</t>
         </is>
       </c>
       <c r="G25" s="8" t="n">
@@ -1641,17 +1633,13 @@
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Дизайнер · имя н/д</t>
-        </is>
-      </c>
-      <c r="G26" s="10" t="n">
-        <v>940000</v>
-      </c>
-      <c r="H26" s="9" t="inlineStr">
-        <is>
-          <t>макс.</t>
-        </is>
-      </c>
+          <t>Ахметова Раушан Нұрланқызы</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="n">
+        <v>815000</v>
+      </c>
+      <c r="H26" s="9" t="inlineStr"/>
       <c r="I26" s="9" t="inlineStr"/>
       <c r="J26" s="5" t="inlineStr">
         <is>
@@ -1685,7 +1673,7 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Дизайнер · имя н/д</t>
+          <t>Ли Яна Вячеславовна</t>
         </is>
       </c>
       <c r="G27" s="10" t="n">
@@ -1729,17 +1717,13 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>Дизайнер · имя н/д</t>
-        </is>
-      </c>
-      <c r="G28" s="10" t="n">
-        <v>940000</v>
-      </c>
-      <c r="H28" s="9" t="inlineStr">
-        <is>
-          <t>макс.</t>
-        </is>
-      </c>
+          <t>Аркениязов Ильяс Юлдашевич</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="n">
+        <v>678061</v>
+      </c>
+      <c r="H28" s="9" t="inlineStr"/>
       <c r="I28" s="9" t="inlineStr"/>
       <c r="J28" s="5" t="inlineStr">
         <is>
@@ -1768,16 +1752,16 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Motion</t>
+          <t>Graph</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Motion-дизайнер · имя н/д</t>
+          <t>Граф дизайнер</t>
         </is>
       </c>
       <c r="G29" s="10" t="n">
-        <v>877000</v>
+        <v>940000</v>
       </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
@@ -1817,17 +1801,13 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>Motion-дизайнер · имя н/д</t>
-        </is>
-      </c>
-      <c r="G30" s="10" t="n">
+          <t>Мкпо Майкл Жозеф</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="n">
         <v>877000</v>
       </c>
-      <c r="H30" s="9" t="inlineStr">
-        <is>
-          <t>макс.</t>
-        </is>
-      </c>
+      <c r="H30" s="9" t="inlineStr"/>
       <c r="I30" s="9" t="inlineStr"/>
       <c r="J30" s="5" t="inlineStr">
         <is>
@@ -1861,7 +1841,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Асанов Әділ · Originals</t>
+          <t>Асанов Әділ Асанұлы</t>
         </is>
       </c>
       <c r="G31" s="8" t="n">
@@ -1901,7 +1881,7 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>Шаймардан Мағжан · Originals</t>
+          <t>Шаймардан Мағжан Адилұлы</t>
         </is>
       </c>
       <c r="G32" s="8" t="n">
@@ -1941,7 +1921,7 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Жұмағали Әділжан · Sport</t>
+          <t>Жұмағали Әділжан Бауыржанұлы</t>
         </is>
       </c>
       <c r="G33" s="8" t="n">
@@ -1961,37 +1941,37 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Проджект</t>
+          <t>Продакшн</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Руководитель</t>
+          <t>Продакшн</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Руководитель</t>
+          <t>Сотрудник</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Head · Ольга М</t>
+          <t>Мобилограф / монтажёр Sport</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>Head project</t>
+          <t>Жанабеков Кудайберген Канатович</t>
         </is>
       </c>
       <c r="G34" s="8" t="n">
-        <v>1291685</v>
+        <v>1498769</v>
       </c>
       <c r="H34" s="9" t="inlineStr"/>
       <c r="I34" s="9" t="inlineStr"/>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>PJ_HEAD</t>
+          <t>P_PROD_4</t>
         </is>
       </c>
     </row>
@@ -2006,32 +1986,32 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Руководитель</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Сотрудник</t>
+          <t>Руководитель</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Project manager · Аружан С</t>
+          <t>Head · Ольга М</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Проджект-менеджер</t>
+          <t>Head project</t>
         </is>
       </c>
       <c r="G35" s="8" t="n">
-        <v>700000</v>
+        <v>1291685</v>
       </c>
       <c r="H35" s="9" t="inlineStr"/>
       <c r="I35" s="9" t="inlineStr"/>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>PJ_1</t>
+          <t>PJ_HEAD</t>
         </is>
       </c>
     </row>
@@ -2056,22 +2036,22 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Project manager · Анель</t>
+          <t>Project manager · Аружан С</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>Муханова Анель Султановна</t>
+          <t>Проджект-менеджер</t>
         </is>
       </c>
       <c r="G36" s="8" t="n">
-        <v>741192</v>
+        <v>700000</v>
       </c>
       <c r="H36" s="9" t="inlineStr"/>
       <c r="I36" s="9" t="inlineStr"/>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>PJ_2</t>
+          <t>PJ_1</t>
         </is>
       </c>
     </row>
@@ -2096,22 +2076,22 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Спецпроекты · Марина</t>
+          <t>Project manager · Анель</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Гяурова Марина Якубовна</t>
+          <t>Муханова Анель Султановна</t>
         </is>
       </c>
       <c r="G37" s="8" t="n">
-        <v>1000162</v>
+        <v>741192</v>
       </c>
       <c r="H37" s="9" t="inlineStr"/>
       <c r="I37" s="9" t="inlineStr"/>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>PJ_3</t>
+          <t>PJ_2</t>
         </is>
       </c>
     </row>
@@ -2136,27 +2116,67 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>B2B и продакшн · Олеся М</t>
+          <t>Спецпроекты · Марина</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>B2B и продакшн</t>
+          <t>Гяурова Марина Якубовна</t>
         </is>
       </c>
       <c r="G38" s="8" t="n">
-        <v>1081000</v>
+        <v>1000162</v>
       </c>
       <c r="H38" s="9" t="inlineStr"/>
       <c r="I38" s="9" t="inlineStr"/>
       <c r="J38" s="5" t="inlineStr">
         <is>
+          <t>PJ_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Проджект</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Сотрудник</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>B2B и продакшн · Олеся М</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>B2B и продакшн</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="n">
+        <v>1081000</v>
+      </c>
+      <c r="H39" s="9" t="inlineStr"/>
+      <c r="I39" s="9" t="inlineStr"/>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
           <t>PJ_4</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="18" t="inlineStr">
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="18" t="inlineStr">
         <is>
           <t>Синие ячейки в «Оклад, ₸» — редактируемые. «Признак: макс.» — имя на позиции не определено, подставлена максимальная стоимость по позиции. «Вакансия: да» — планируемая позиция. Итоги считаются на листе «Свод».</t>
         </is>
@@ -2164,8 +2184,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A40:J40"/>
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A41:J41"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2216,11 +2236,11 @@
         </is>
       </c>
       <c r="B3" s="22">
-        <f>COUNTIF(Данные!$B$3:$B$38,A3)</f>
+        <f>COUNTIF(Данные!$B$3:$B$39,A3)</f>
         <v/>
       </c>
       <c r="C3" s="23">
-        <f>SUMIF(Данные!$B$3:$B$38,A3,Данные!$G$3:$G$38)</f>
+        <f>SUMIF(Данные!$B$3:$B$39,A3,Данные!$G$3:$G$39)</f>
         <v/>
       </c>
     </row>
@@ -2231,11 +2251,11 @@
         </is>
       </c>
       <c r="B4" s="25">
-        <f>COUNTIF(Данные!$B$3:$B$38,A4)</f>
+        <f>COUNTIF(Данные!$B$3:$B$39,A4)</f>
         <v/>
       </c>
       <c r="C4" s="26">
-        <f>SUMIF(Данные!$B$3:$B$38,A4,Данные!$G$3:$G$38)</f>
+        <f>SUMIF(Данные!$B$3:$B$39,A4,Данные!$G$3:$G$39)</f>
         <v/>
       </c>
     </row>
@@ -2246,11 +2266,11 @@
         </is>
       </c>
       <c r="B5" s="22">
-        <f>COUNTIF(Данные!$B$3:$B$38,A5)</f>
+        <f>COUNTIF(Данные!$B$3:$B$39,A5)</f>
         <v/>
       </c>
       <c r="C5" s="23">
-        <f>SUMIF(Данные!$B$3:$B$38,A5,Данные!$G$3:$G$38)</f>
+        <f>SUMIF(Данные!$B$3:$B$39,A5,Данные!$G$3:$G$39)</f>
         <v/>
       </c>
     </row>
@@ -2261,11 +2281,11 @@
         </is>
       </c>
       <c r="B6" s="25">
-        <f>COUNTIF(Данные!$B$3:$B$38,A6)</f>
+        <f>COUNTIF(Данные!$B$3:$B$39,A6)</f>
         <v/>
       </c>
       <c r="C6" s="26">
-        <f>SUMIF(Данные!$B$3:$B$38,A6,Данные!$G$3:$G$38)</f>
+        <f>SUMIF(Данные!$B$3:$B$39,A6,Данные!$G$3:$G$39)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Leave the fourth Graph position empty (open role, 940 000 ₸ *)
Clear the «Граф дизайнер» placeholder name per request; the box stays an
open Graph position with the max cost 940 000 ₸ and its * marker. The
existing * markers on the named SMM/Graph rows are kept as-is. Totals
unchanged (Продакшн 13 581 877 ₸, grand 41 605 842 ₸).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015FvdqNtbbJPjugTChUgZkw
</commit_message>
<xml_diff>
--- a/Данные — структура и ФОТ.xlsx
+++ b/Данные — структура и ФОТ.xlsx
@@ -1755,11 +1755,7 @@
           <t>Graph</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>Граф дизайнер</t>
-        </is>
-      </c>
+      <c r="F29" s="7" t="inlineStr"/>
       <c r="G29" s="10" t="n">
         <v>940000</v>
       </c>

</xml_diff>